<commit_message>
Remove nonbusiness data provenance wording
</commit_message>
<xml_diff>
--- a/artifacts/关键标准答案.xlsx
+++ b/artifacts/关键标准答案.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="R5c21894547eb463d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="R251c35890b394d41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="R4caf4888e4f74dfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="Rfcc80752f5634eb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="Ra9ff92d991cd4524"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="R3b8d101c64c44b61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="R18f42f3145cd4831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="Rf68717c7ed714d67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="Rbb71970caff64afa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="R3850d4978b474311"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -672,7 +672,7 @@
         <x:v>PodSpec中的镜像与ServiceAccount</x:v>
       </x:c>
       <x:c r="C4" s="24" t="str">
-        <x:v>由values.yaml合成</x:v>
+        <x:v>与values.yaml中的镜像及服务账号字段一致</x:v>
       </x:c>
       <x:c r="D4" s="25" t="str">
         <x:v>values.yaml</x:v>

</xml_diff>